<commit_message>
Long method files are added before analysis!
</commit_message>
<xml_diff>
--- a/util/Validation/ManualValidation/largeClassForManual.xlsx
+++ b/util/Validation/ManualValidation/largeClassForManual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Desktop/workspace/BadSmells/util/Validation/ManualValidation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Documents/workspace/DissertationProject/util/Validation/ManualValidation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2B2BF5-CE43-B545-88F3-CD1BBF35344A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7988731A-B118-A54A-BBDE-392D732959D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="23640" windowHeight="14520" xr2:uid="{3004C773-7DF2-304E-B74E-6C331540559A}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="23640" windowHeight="14200" xr2:uid="{3004C773-7DF2-304E-B74E-6C331540559A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$F$1:$F$642</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$640</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3970,7 +3970,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>77</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>86</v>
       </c>
@@ -4905,7 +4905,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>135</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>139</v>
       </c>
@@ -5040,7 +5040,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
         <v>780</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>140</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>146</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
         <v>169</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
         <v>200</v>
       </c>
@@ -8206,7 +8206,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" s="2" t="s">
         <v>277</v>
       </c>
@@ -8233,7 +8233,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" s="2" t="s">
         <v>279</v>
       </c>
@@ -8314,7 +8314,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" s="2" t="s">
         <v>285</v>
       </c>
@@ -8422,7 +8422,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" s="2" t="s">
         <v>292</v>
       </c>
@@ -8692,7 +8692,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" s="2" t="s">
         <v>310</v>
       </c>
@@ -10725,7 +10725,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="368" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A368" s="2" t="s">
         <v>453</v>
       </c>
@@ -11548,7 +11548,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="402" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A402" s="2" t="s">
         <v>494</v>
       </c>
@@ -11899,7 +11899,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="415" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A415" s="2" t="s">
         <v>509</v>
       </c>
@@ -11934,7 +11934,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="417" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A417" s="2" t="s">
         <v>512</v>
       </c>
@@ -12028,7 +12028,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="424" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="424" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A424" s="2" t="s">
         <v>521</v>
       </c>
@@ -16295,7 +16295,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="629" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="629" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A629" s="2" t="s">
         <v>781</v>
       </c>
@@ -16430,7 +16430,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="634" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="634" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A634" t="s">
         <v>765</v>
       </c>
@@ -16457,7 +16457,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="635" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="635" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A635" t="s">
         <v>766</v>
       </c>
@@ -16600,17 +16600,17 @@
         <v>772</v>
       </c>
     </row>
-    <row r="641" spans="9:9" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="642" spans="9:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="642" spans="9:9" x14ac:dyDescent="0.2">
       <c r="I642">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="F1:F642" xr:uid="{2472F359-1722-2740-8C96-A1C26FFBD658}">
+  <autoFilter ref="A1:I640" xr:uid="{CA9CF15E-E3A6-1B49-8A2A-5F0F2EDE25DD}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Yes"/>
+        <filter val="TemplateObject"/>
+        <filter val="TemplateObjectGetter"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>